<commit_message>
update 1 file and delete 7 files
</commit_message>
<xml_diff>
--- a/excel/Healthy_Lifestyle.xlsx
+++ b/excel/Healthy_Lifestyle.xlsx
@@ -16,14 +16,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
   <si>
     <t>Wake Up Early</t>
   </si>
   <si>
-    <t>Learn Something New</t>
-  </si>
-  <si>
     <t>Workout</t>
   </si>
   <si>
@@ -60,61 +57,73 @@
     <t>English Communication</t>
   </si>
   <si>
-    <t>6 June, 2025</t>
-  </si>
-  <si>
-    <t>7 June, 2025</t>
-  </si>
-  <si>
-    <t>8 June, 2025</t>
-  </si>
-  <si>
-    <t>9 June, 2025</t>
-  </si>
-  <si>
-    <t>10 June, 2025</t>
-  </si>
-  <si>
-    <t>11 June, 2025</t>
-  </si>
-  <si>
-    <t>12 June, 2025</t>
-  </si>
-  <si>
-    <t>13 June, 2025</t>
-  </si>
-  <si>
-    <t>14 June, 2025</t>
-  </si>
-  <si>
-    <t>15 June, 2025</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
     <t>✅</t>
   </si>
   <si>
-    <t>16 June, 2025</t>
-  </si>
-  <si>
-    <t>17 June, 2025</t>
-  </si>
-  <si>
-    <t>18 June, 2025</t>
-  </si>
-  <si>
-    <t>19 June, 2025</t>
-  </si>
-  <si>
-    <t>20 June, 2025</t>
-  </si>
-  <si>
-    <t>21 June, 2025</t>
-  </si>
-  <si>
-    <t>22 June, 2025</t>
+    <t>6 Jun, 2025</t>
+  </si>
+  <si>
+    <t>7 Jun, 2025</t>
+  </si>
+  <si>
+    <t>8 Jun, 2025</t>
+  </si>
+  <si>
+    <t>9 Jun, 2025</t>
+  </si>
+  <si>
+    <t>10 Jun, 2025</t>
+  </si>
+  <si>
+    <t>11 Jun, 2025</t>
+  </si>
+  <si>
+    <t>12 Jun, 2025</t>
+  </si>
+  <si>
+    <t>13 Jun, 2025</t>
+  </si>
+  <si>
+    <t>14 Jun, 2025</t>
+  </si>
+  <si>
+    <t>15 Jun, 2025</t>
+  </si>
+  <si>
+    <t>16 Jun, 2025</t>
+  </si>
+  <si>
+    <t>17 Jun, 2025</t>
+  </si>
+  <si>
+    <t>18 Jun, 2025</t>
+  </si>
+  <si>
+    <t>19 Jun, 2025</t>
+  </si>
+  <si>
+    <t>20 Jun, 2025</t>
+  </si>
+  <si>
+    <t>21 Jun, 2025</t>
+  </si>
+  <si>
+    <t>22 Jun, 2025</t>
+  </si>
+  <si>
+    <t>23 Jun, 2025</t>
+  </si>
+  <si>
+    <t>No Phone 1st 30 min</t>
+  </si>
+  <si>
+    <t>No Phone After 10.30 pm</t>
+  </si>
+  <si>
+    <t>Learn Something New (P/P)</t>
   </si>
 </sst>
 </file>
@@ -260,7 +269,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -287,6 +296,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -588,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.85546875" customWidth="1"/>
@@ -597,72 +609,84 @@
     <col min="4" max="4" width="18.42578125" customWidth="1"/>
     <col min="5" max="5" width="10.140625" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="22.85546875" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="14.85546875" customWidth="1"/>
     <col min="9" max="9" width="18.140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" customWidth="1"/>
     <col min="12" max="12" width="12.5703125" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="14" max="14" width="19.5703125" customWidth="1"/>
+    <col min="15" max="15" width="23.5703125" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="C2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>14</v>
+      </c>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
@@ -674,9 +698,9 @@
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:17">
       <c r="A3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -692,9 +716,9 @@
       <c r="M3" s="6"/>
       <c r="N3" s="6"/>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:17">
       <c r="A4" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -710,9 +734,9 @@
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:17">
       <c r="A5" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -728,9 +752,9 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:17">
       <c r="A6" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -746,9 +770,9 @@
       <c r="M6" s="6"/>
       <c r="N6" s="6"/>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:17">
       <c r="A7" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -764,9 +788,9 @@
       <c r="M7" s="6"/>
       <c r="N7" s="6"/>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:17">
       <c r="A8" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -782,9 +806,9 @@
       <c r="M8" s="6"/>
       <c r="N8" s="6"/>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:17">
       <c r="A9" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -800,9 +824,9 @@
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:17">
       <c r="A10" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -818,9 +842,9 @@
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:17">
       <c r="A11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -836,38 +860,43 @@
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:17">
       <c r="A12" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17">
+      <c r="A13" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="5" t="s">
+    <row r="14" spans="1:17">
+      <c r="A14" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="5" t="s">
+    <row r="15" spans="1:17">
+      <c r="A15" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="5" t="s">
+    <row r="16" spans="1:17">
+      <c r="A16" s="5" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="5" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update Healthy_Lifestyle.xlsx and weight_loss_plan.xlsx
</commit_message>
<xml_diff>
--- a/excel/Healthy_Lifestyle.xlsx
+++ b/excel/Healthy_Lifestyle.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="38">
   <si>
     <t>Wake Up Early</t>
   </si>
@@ -800,37 +800,107 @@
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
+      <c r="B4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" s="9" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
+      <c r="B5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="5" t="s">

</xml_diff>

<commit_message>
update Healthy_Lifestyle.xlsx and day_routine.xlsx
</commit_message>
<xml_diff>
--- a/excel/Healthy_Lifestyle.xlsx
+++ b/excel/Healthy_Lifestyle.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="38">
   <si>
     <t>Wake Up Early</t>
   </si>
@@ -136,7 +136,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -179,13 +179,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Wingdings"/>
-      <charset val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -282,7 +275,7 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="4" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -302,19 +295,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -680,13 +670,13 @@
       <c r="N1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="O1" s="9" t="s">
         <v>36</v>
       </c>
       <c r="P1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -694,52 +684,52 @@
       <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="M2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="O2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="P2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q2" s="9" t="s">
+      <c r="B2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -747,52 +737,52 @@
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="M3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="N3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="P3" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q3" s="9" t="s">
+      <c r="B3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -800,52 +790,52 @@
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="P4" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q4" s="9" t="s">
+      <c r="B4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q4" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -853,52 +843,52 @@
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="L5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="N5" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="P5" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" s="9" t="s">
+      <c r="B5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q5" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -906,19 +896,54 @@
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
+      <c r="B6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q6" s="8" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="7" spans="1:17">
       <c r="A7" s="5" t="s">

</xml_diff>